<commit_message>
Aggiornamento dati reali da pulsante iPhone
</commit_message>
<xml_diff>
--- a/Database_App_Betting.xlsx
+++ b/Database_App_Betting.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,162 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Goal_NoGoal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FIFA World Cup</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>16/06/2026 17:19</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Argentina - Francia</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FIFA World Cup</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>16/06/2026 17:19</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Italia - Stati Uniti</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FIFA World Cup</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>16/06/2026 17:19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Brasile - Giappone</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>In elaborazione</t>
         </is>
       </c>
     </row>

</xml_diff>